<commit_message>
W1-05: sort cleaning decisions into approved, disputed and unresolved
- Re-status all 33 decisions by evidence type: 15 approved, 5 disputed
  (D05-D08, C04), 13 unresolved (D17-D29: follicle count 0 with a
  recorded size; raw values kept, to be flagged).
- Add evidence_type, reference and sensitivity_variant columns, with
  peer-reviewed 2020-2026 references for the physiological thresholds.
- D14-D16 (zero placeholders) treated as verifiable from the record.
- No rows remain 'proposed', so the current code applies only approved
  decisions.
- Remove template instructions and colour coding.
</commit_message>
<xml_diff>
--- a/docs/cleaning_decisions.xlsx
+++ b/docs/cleaning_decisions.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decisions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'decisions'!$A$4:$J$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'decisions'!$A$4:$M$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +48,15 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="4">
@@ -94,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -108,6 +117,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -486,19 +497,22 @@
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="70" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Cleaning decisions (read by src/preprocessing.py)</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Cleaning decisions</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Status: proposed = applied for now, still to agree with supervisor | approved = agreed, applied | rejected = not applied. Change status or action in the yellow cells, then rerun notebook 05.</t>
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Status: approved = applied | disputed = not applied until the supervisor agrees | unresolved = not applied, raw value kept and flagged | rejected = never applied.</t>
         </is>
       </c>
     </row>
@@ -553,6 +567,21 @@
           <t>source</t>
         </is>
       </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>evidence_type</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>sensitivity_variant</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -578,15 +607,15 @@
           <t>18</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -599,6 +628,17 @@
           <t>IMP-04</t>
         </is>
       </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>B - outside cited physiological range</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Quer G, Gouda P, Galarnyk M, Topol EJ, Steinhubl SR (2020). Inter- and intraindividual variability in daily resting heart rate... 92,457 adults. PLoS One 15(2):e0227709. doi:10.1371/journal.pone.0227709 (individual mean resting HR 40-109 bpm).</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -624,15 +664,15 @@
           <t>13</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
@@ -645,6 +685,17 @@
           <t>IMP-04</t>
         </is>
       </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>B - outside cited physiological range</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Quer G, Gouda P, Galarnyk M, Topol EJ, Steinhubl SR (2020). Inter- and intraindividual variability in daily resting heart rate... 92,457 adults. PLoS One 15(2):e0227709. doi:10.1371/journal.pone.0227709 (individual mean resting HR 40-109 bpm).</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -670,15 +721,15 @@
           <t>12</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -691,6 +742,17 @@
           <t>IMP-04</t>
         </is>
       </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>B - outside cited physiological range</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>McEvoy JW, ..., Touyz RM; ESC Scientific Document Group (2024). 2024 ESC Guidelines for the management of elevated blood pressure and hypertension. Eur Heart J 45(38):3912-4018. doi:10.1093/eurheartj/ehae178 (non-elevated BP &lt;120/&lt;70 mmHg; values of 12 and 8 are an order of magnitude below any category).</t>
+        </is>
+      </c>
+      <c r="M7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -716,15 +778,15 @@
           <t>8</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -737,6 +799,17 @@
           <t>IMP-04</t>
         </is>
       </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>B - outside cited physiological range</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>McEvoy JW, ..., Touyz RM; ESC Scientific Document Group (2024). 2024 ESC Guidelines for the management of elevated blood pressure and hypertension. Eur Heart J 45(38):3912-4018. doi:10.1093/eurheartj/ehae178 (non-elevated BP &lt;120/&lt;70 mmHg; values of 12 and 8 are an order of magnitude below any category).</t>
+        </is>
+      </c>
+      <c r="M8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -762,15 +835,15 @@
           <t>5052</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>disputed</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -781,6 +854,21 @@
       <c r="J9" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>B - outside cited physiological range</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Kawakita T, Yasui T, Yoshida K, Matsui S, ..., Iwasa T (2023). Associations of LH and FSH with reproductive hormones depending on each stage of the menopausal transition. BMC Womens Health 23:286. doi:10.1186/s12905-023-02438-5 (highest median FSH 95.85 mIU/mL, upper quartile 123.7; LH plateaus at median 33.3, upper quartile 43.9, in early postmenopause).</t>
+        </is>
+      </c>
+      <c r="M9" s="6" t="inlineStr">
+        <is>
+          <t>Compare results with and without the correction.</t>
         </is>
       </c>
     </row>
@@ -808,15 +896,15 @@
           <t>2018</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>disputed</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
@@ -827,6 +915,21 @@
       <c r="J10" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>B - outside cited physiological range</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Kawakita T, Yasui T, Yoshida K, Matsui S, ..., Iwasa T (2023). Associations of LH and FSH with reproductive hormones depending on each stage of the menopausal transition. BMC Womens Health 23:286. doi:10.1186/s12905-023-02438-5 (highest median FSH 95.85 mIU/mL, upper quartile 123.7; LH plateaus at median 33.3, upper quartile 43.9, in early postmenopause).</t>
+        </is>
+      </c>
+      <c r="M10" s="6" t="inlineStr">
+        <is>
+          <t>Compare results with and without the correction.</t>
         </is>
       </c>
     </row>
@@ -854,15 +957,15 @@
           <t>6014.66</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>disputed</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -873,6 +976,21 @@
       <c r="J11" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>B - outside cited physiological range</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Fabregat-Bolufer AB, Martin-Alonso C, Escola-Rodriguez A, Morales-Ruiz M (2026). Overdiagnosed and oversupplemented: the iatrogenic rise of vitamin D toxicity. Eur J Endocrinol 194(6):K21. doi:10.1093/ejendo/lvag088 (&gt;100 ng/mL treated as very high / hypervitaminosis D).</t>
+        </is>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>Compare results with and without the correction.</t>
         </is>
       </c>
     </row>
@@ -900,15 +1018,15 @@
           <t>5418.6</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>disputed</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
@@ -919,6 +1037,21 @@
       <c r="J12" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>B - outside cited physiological range</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>Fabregat-Bolufer AB, Martin-Alonso C, Escola-Rodriguez A, Morales-Ruiz M (2026). Overdiagnosed and oversupplemented: the iatrogenic rise of vitamin D toxicity. Eur J Endocrinol 194(6):K21. doi:10.1093/ejendo/lvag088 (&gt;100 ng/mL treated as very high / hypervitaminosis D).</t>
+        </is>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>Compare results with and without the correction.</t>
         </is>
       </c>
     </row>
@@ -946,15 +1079,15 @@
           <t>66</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>keep</t>
         </is>
       </c>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -965,6 +1098,21 @@
       <c r="J13" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>C - keep (no data change)</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>Nguyen MT, Krishnan S, Phatak SV, Karakas SE (2023). Anti-Mullerian hormone-based phenotyping identifies subgroups of women with PCOS... Diagnostics 13(3):500. doi:10.3390/diagnostics13030500 (highest AMH quartile 18.5 +/- 9.9 ng/mL). Schwenck-Carvalho PJ et al. (2026). AMH levels across phenotypes in PCOS: systematic review and meta-analysis. J Endocr Soc 10(3). doi:10.1210/jendso/bvaf199.</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
+          <t>Influence check: refit without this record.</t>
         </is>
       </c>
     </row>
@@ -992,15 +1140,15 @@
           <t>5</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1013,6 +1161,13 @@
           <t>IMP-04</t>
         </is>
       </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>A - verifiable from record</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr"/>
+      <c r="M14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1038,15 +1193,15 @@
           <t>20.3</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>recompute</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -1059,6 +1214,13 @@
           <t>IMP-04</t>
         </is>
       </c>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>A - verifiable from record</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr"/>
+      <c r="M15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1084,19 +1246,19 @@
           <t>'1.99.'</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>correct</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>1.99</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
@@ -1109,6 +1271,13 @@
           <t>IMP-03/04</t>
         </is>
       </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>A - verifiable from record</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr"/>
+      <c r="M16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1134,15 +1303,15 @@
           <t>'a'</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -1155,6 +1324,13 @@
           <t>IMP-03</t>
         </is>
       </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>A - verifiable from record</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1180,20 +1356,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Impossible zero: a measured vitamin D level cannot be 0.</t>
+          <t>Zero is not a possible vitamin D measurement, so it is a placeholder for 'not measured'; set to missing.</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1201,6 +1377,13 @@
           <t>IMP-03</t>
         </is>
       </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>A - verifiable from record</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr"/>
+      <c r="M18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1226,20 +1409,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Impossible zero: endometrial thickness cannot be 0 mm.</t>
+          <t>Zero is not a possible endometrial thickness measurement, so it is a placeholder for 'not measured'; set to missing.</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1247,6 +1430,13 @@
           <t>IMP-03</t>
         </is>
       </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>A - verifiable from record</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr"/>
+      <c r="M19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1272,20 +1462,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Impossible zero: endometrial thickness cannot be 0 mm.</t>
+          <t>Zero is not a possible endometrial thickness measurement, so it is a placeholder for 'not measured'; set to missing.</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1293,6 +1483,13 @@
           <t>IMP-03</t>
         </is>
       </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>A - verifiable from record</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr"/>
+      <c r="M20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1318,25 +1515,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 15 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 15 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr"/>
+      <c r="M21" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1364,25 +1572,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 17 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 17 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr"/>
+      <c r="M22" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1410,25 +1629,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 17 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 17 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr"/>
+      <c r="M23" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1456,25 +1686,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 15 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 15 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="inlineStr"/>
+      <c r="M24" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1502,25 +1743,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 20 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 20 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="inlineStr"/>
+      <c r="M25" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1548,25 +1800,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 18 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 18 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L26" s="6" t="inlineStr"/>
+      <c r="M26" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1594,25 +1857,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 12 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 12 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L27" s="6" t="inlineStr"/>
+      <c r="M27" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1640,25 +1914,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 18 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 18 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L28" s="6" t="inlineStr"/>
+      <c r="M28" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1686,25 +1971,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 11 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 11 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="inlineStr"/>
+      <c r="M29" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1732,25 +2028,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 14 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 14 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="inlineStr"/>
+      <c r="M30" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1778,25 +2085,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 16 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 16 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K31" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L31" s="6" t="inlineStr"/>
+      <c r="M31" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1824,25 +2142,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 10 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 10 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr"/>
+      <c r="M32" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1870,25 +2199,36 @@
           <t>0</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>set_missing</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>set_missing</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="n"/>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>unresolved</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>Count 0 contradicts an average follicle size of 9 mm; a recorded size implies follicles were seen, so the count is distrusted.</t>
+          <t>Count 0 contradicts an average follicle size of 9 mm. The record does not show which field is wrong (count, size, or a recording convention), so neither is changed; the record is flagged instead.</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
           <t>IMP-04</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>D - contradictory record</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr"/>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>Raw value kept and flagged (follicle_inconsistent). Compare (i) raw values, (ii) count set to missing, (iii) count and size set to missing.</t>
         </is>
       </c>
     </row>
@@ -1910,19 +2250,19 @@
         </is>
       </c>
       <c r="E34" s="4" t="n"/>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>recompute</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>FSH / LH</t>
         </is>
       </c>
-      <c r="H34" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
@@ -1935,6 +2275,13 @@
           <t>IMP-04</t>
         </is>
       </c>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>A - verifiable from record</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="inlineStr"/>
+      <c r="M34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1958,19 +2305,19 @@
           <t>2 / 4</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>recode</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>2=0, 4=1</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -1983,6 +2330,13 @@
           <t>IMP-05</t>
         </is>
       </c>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>A - verifiable from record</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr"/>
+      <c r="M35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2006,15 +2360,15 @@
           <t>highlighted cells</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>keep</t>
         </is>
       </c>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2027,6 +2381,13 @@
           <t>IMP-03</t>
         </is>
       </c>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>C - keep (no data change)</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr"/>
+      <c r="M36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2050,15 +2411,15 @@
           <t>1.99</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>keep</t>
         </is>
       </c>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>proposed</t>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>disputed</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -2071,15 +2432,33 @@
           <t>IMP-03</t>
         </is>
       </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>C - keep (no data change)</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>Ortega-Villa AM, Liu D, Ward MH, Albert PS (2021). New insights into modeling exposure measurements below the limit of detection. Environ Epidemiol 5(1):e116. doi:10.1097/EE9.0000000000000116 (substitution can bias estimates even when &lt;20% of values are below the limit).</t>
+        </is>
+      </c>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>Compare (i) 1.99 kept as a value, (ii) 1.99 treated as below the detection limit with a flag, (iii) 1.99 set to missing.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J37"/>
-  <dataValidations count="2">
+  <autoFilter ref="A4:M37"/>
+  <dataValidations count="3">
     <dataValidation sqref="F5:F67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"set_missing,correct,recompute,recode,keep"</formula1>
     </dataValidation>
     <dataValidation sqref="H5:H67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"proposed,approved,rejected"</formula1>
+      <formula1>"approved,disputed,unresolved,rejected"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K5:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"A - verifiable from record,B - outside cited physiological range,C - keep (no data change),D - contradictory record"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
C03: record highlighted vitamin D values as source-marked manipulated
The official Kaggle instructions say manipulated values were highlighted
in an orangish colour. C03 keeps the 22 highlighted values (status
approved, action keep), reports them as a limitation and adds a
sensitivity variant (kept vs set to missing).
</commit_message>
<xml_diff>
--- a/docs/cleaning_decisions.xlsx
+++ b/docs/cleaning_decisions.xlsx
@@ -2373,12 +2373,12 @@
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>22 reddish-highlighted values (patients 307-328) may have been filled in; meaning unconfirmed, so kept and reported as a limitation.</t>
+          <t>22 highlighted values (patients 307-328) are values the source marked as manipulated: the official Kaggle instructions say manipulated data were highlighted in an orangish colour. Kept, reported as a limitation, and tested in a sensitivity analysis.</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>IMP-03</t>
+          <t>IMP-03; Kaggle dataset page (official instructions)</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
@@ -2387,7 +2387,11 @@
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr"/>
-      <c r="M36" s="6" t="inlineStr"/>
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>Compare (i) highlighted values kept, (ii) highlighted values set to missing.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">

</xml_diff>